<commit_message>
Widen annual tolerance band; add extract_frequency_key for future per-amount split
- frequency_lookup.py: ANNUAL_MAX_DAYS 400 -> 430 to allow for renewal-date drift
- vendor_lookup.py: new extract_frequency_key() -- additive, doesn't change account-code lookup
- Diagnosed real cause of Apple/Microsoft/GoDaddy frequency misclassification:
  multiple distinct recurring charges collapsed under one vendor name.
  Not fully fixed yet -- needs an amount-based split, documented in the guide's Known Issues section.
</commit_message>
<xml_diff>
--- a/historical_vendor_database.xlsx
+++ b/historical_vendor_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E399"/>
+  <dimension ref="A1:E402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10393,6 +10393,81 @@
         </is>
       </c>
     </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>HOTEL ALEX JOHNSON RRAPID CITY</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>80.21.05</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>G&amp;A Travel</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>1</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Promoted from review</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>ENTERPRISE RENT-A-CARAPID CITY</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>80.21.05</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>G&amp;A Travel</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>1</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Promoted from review</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>TST* LA PARISIENNE 0NEW YORK</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>80.21.11</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>G&amp;A Meals</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>1</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Promoted from review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>